<commit_message>
minor edits to plots
</commit_message>
<xml_diff>
--- a/data/ASP_input_parameters_german2.xlsx
+++ b/data/ASP_input_parameters_german2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prajna\Documents\HORTIBONN\PROJECTS\Onion_DA_model\hotri_bonn_Repo\Climate_Impact_on_Crop_Yield\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C8E9587-4EAB-41D0-862E-A81C6E25A3C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{400C0F09-134A-405D-BA45-D0717A427AB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-2325" windowWidth="38640" windowHeight="21120" tabRatio="815" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-2325" windowWidth="38640" windowHeight="21120" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet_names" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="310">
   <si>
     <t>variable</t>
   </si>
@@ -592,18 +592,6 @@
     <t>Gewichtungsfaktor (0–1), der angibt, wie stark aufeinanderfolgende Tage mit günstigen Bedingungen für Hagel das Risiko beeinflussen.</t>
   </si>
   <si>
-    <t>latitude_koeln_bonn_c</t>
-  </si>
-  <si>
-    <t>Latitude [°N]</t>
-  </si>
-  <si>
-    <t>Breitengrad von Köln Bonn (Referenzort)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zwiebelbauer;Zwiebel Anbauberater;Datenanalyst </t>
-  </si>
-  <si>
     <t>HI_onions_t</t>
   </si>
   <si>
@@ -628,15 +616,6 @@
     <t>Spagelbauer;Datenanalyst;Market analyst;Policy-maker</t>
   </si>
   <si>
-    <t>rain_window_days_sowing_p</t>
-  </si>
-  <si>
-    <t>Rainfall window before sowing [days]</t>
-  </si>
-  <si>
-    <t>The number of days before sowing is considered for the rainfall accumulation check.</t>
-  </si>
-  <si>
     <t>leaf_area_em_per_plant_p</t>
   </si>
   <si>
@@ -988,10 +967,10 @@
     <t>Bestimmt, wie leer das pflanzenverfügbare Bodenwasserreservoir sein darf, bevor eine Bewässerung ausgelöst wird. Ein Wert von 0,5 bedeutet: Sobald die Hälfte des nutzbaren Wassers verbraucht ist, wird bewässert.</t>
   </si>
   <si>
-    <t>Bodenparameter</t>
-  </si>
-  <si>
     <t>slider1</t>
+  </si>
+  <si>
+    <t>Bewässerungsparameter</t>
   </si>
 </sst>
 </file>
@@ -1468,7 +1447,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="B8" t="s">
         <v>9</v>
@@ -1574,10 +1553,10 @@
         <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="K2" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1609,10 +1588,10 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="K3" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1644,10 +1623,10 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="K4" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:11" s="1" customFormat="1">
@@ -1679,10 +1658,10 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="K5" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:11" s="1" customFormat="1">
@@ -1714,15 +1693,15 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="K6" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="B7" s="15">
         <v>45</v>
@@ -1734,13 +1713,13 @@
         <v>5</v>
       </c>
       <c r="E7" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="F7" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="G7" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="H7" t="s">
         <v>19</v>
@@ -1749,7 +1728,7 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1784,12 +1763,12 @@
         <v>161</v>
       </c>
       <c r="K8" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B9" s="15">
         <v>0.65</v>
@@ -1816,7 +1795,7 @@
         <v>161</v>
       </c>
       <c r="K9" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -1908,10 +1887,10 @@
         <v>0.1</v>
       </c>
       <c r="J2" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="K2" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1943,10 +1922,10 @@
         <v>0.1</v>
       </c>
       <c r="J3" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="K3" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1978,10 +1957,10 @@
         <v>0.1</v>
       </c>
       <c r="J4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="K4" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -2013,10 +1992,10 @@
         <v>0.1</v>
       </c>
       <c r="J5" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="K5" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -2161,10 +2140,10 @@
         <v>0.1</v>
       </c>
       <c r="J2" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="K2" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -2196,10 +2175,10 @@
         <v>0.1</v>
       </c>
       <c r="J3" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="K3" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -2231,10 +2210,10 @@
         <v>0.1</v>
       </c>
       <c r="J4" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="K4" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -2266,10 +2245,10 @@
         <v>0.1</v>
       </c>
       <c r="J5" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="K5" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -2397,7 +2376,7 @@
         <v>76</v>
       </c>
       <c r="K3" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -2432,7 +2411,7 @@
         <v>76</v>
       </c>
       <c r="K4" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -2450,7 +2429,7 @@
       </c>
       <c r="E5"/>
       <c r="F5" s="12" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="G5" s="12" t="s">
         <v>87</v>
@@ -2465,7 +2444,7 @@
         <v>77</v>
       </c>
       <c r="K5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -2483,10 +2462,10 @@
       </c>
       <c r="E6"/>
       <c r="F6" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="G6" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="H6" t="s">
         <v>19</v>
@@ -2498,7 +2477,7 @@
         <v>77</v>
       </c>
       <c r="K6" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -2534,10 +2513,10 @@
         <v>78</v>
       </c>
       <c r="F9" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="G9" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="H9" t="s">
         <v>19</v>
@@ -2549,7 +2528,7 @@
         <v>161</v>
       </c>
       <c r="K9" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -2569,10 +2548,10 @@
         <v>92</v>
       </c>
       <c r="F10" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="G10" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="H10" t="s">
         <v>19</v>
@@ -2584,7 +2563,7 @@
         <v>161</v>
       </c>
       <c r="K10" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -2602,7 +2581,7 @@
       </c>
       <c r="E11"/>
       <c r="F11" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="G11" t="s">
         <v>182</v>
@@ -2617,12 +2596,12 @@
         <v>161</v>
       </c>
       <c r="K11" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B12">
         <v>0.5</v>
@@ -2635,10 +2614,10 @@
       </c>
       <c r="E12"/>
       <c r="F12" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="G12" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="H12" t="s">
         <v>19</v>
@@ -2650,7 +2629,7 @@
         <v>161</v>
       </c>
       <c r="K12" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -2670,7 +2649,7 @@
     </row>
     <row r="15" spans="1:14">
       <c r="A15" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="B15" s="13">
         <v>30</v>
@@ -2685,10 +2664,10 @@
         <v>92</v>
       </c>
       <c r="F15" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="G15" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="H15" t="s">
         <v>19</v>
@@ -2697,10 +2676,10 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K15" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L15"/>
       <c r="M15"/>
@@ -2708,7 +2687,7 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="B16" s="14">
         <v>0.6</v>
@@ -2721,10 +2700,10 @@
       </c>
       <c r="E16"/>
       <c r="F16" s="12" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="G16" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="H16" t="s">
         <v>19</v>
@@ -2733,10 +2712,10 @@
         <v>0.1</v>
       </c>
       <c r="J16" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K16" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L16"/>
       <c r="M16"/>
@@ -2744,7 +2723,7 @@
     </row>
     <row r="17" spans="1:14">
       <c r="A17" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="B17" s="14">
         <v>0.5</v>
@@ -2757,10 +2736,10 @@
       </c>
       <c r="E17"/>
       <c r="F17" s="12" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="G17" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="H17" t="s">
         <v>19</v>
@@ -2769,10 +2748,10 @@
         <v>0.1</v>
       </c>
       <c r="J17" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K17" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L17"/>
       <c r="M17"/>
@@ -2780,7 +2759,7 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="B18" s="14">
         <v>0.05</v>
@@ -2793,10 +2772,10 @@
       </c>
       <c r="E18"/>
       <c r="F18" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="G18" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="H18" t="s">
         <v>19</v>
@@ -2805,10 +2784,10 @@
         <v>0.05</v>
       </c>
       <c r="J18" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K18" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="L18"/>
       <c r="M18"/>
@@ -3006,7 +2985,7 @@
         <v>170</v>
       </c>
       <c r="G3" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="H3" t="s">
         <v>19</v>
@@ -3018,7 +2997,7 @@
         <v>161</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -3041,7 +3020,7 @@
         <v>102</v>
       </c>
       <c r="G4" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="H4" t="s">
         <v>19</v>
@@ -3053,7 +3032,7 @@
         <v>161</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -3076,7 +3055,7 @@
         <v>103</v>
       </c>
       <c r="G5" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="H5" t="s">
         <v>19</v>
@@ -3088,7 +3067,7 @@
         <v>161</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -3109,7 +3088,7 @@
         <v>172</v>
       </c>
       <c r="G6" s="12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H6" t="s">
         <v>19</v>
@@ -3121,7 +3100,7 @@
         <v>161</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -3142,7 +3121,7 @@
         <v>100</v>
       </c>
       <c r="G7" s="12" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="H7" t="s">
         <v>19</v>
@@ -3154,7 +3133,7 @@
         <v>161</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -3175,7 +3154,7 @@
         <v>105</v>
       </c>
       <c r="G8" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="H8" t="s">
         <v>19</v>
@@ -3187,7 +3166,7 @@
         <v>161</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -3222,10 +3201,10 @@
         <v>78</v>
       </c>
       <c r="F11" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="G11" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="H11" t="s">
         <v>19</v>
@@ -3237,7 +3216,7 @@
         <v>161</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -3257,10 +3236,10 @@
         <v>92</v>
       </c>
       <c r="F12" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="G12" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="H12" t="s">
         <v>19</v>
@@ -3272,7 +3251,7 @@
         <v>161</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -3292,10 +3271,10 @@
         <v>92</v>
       </c>
       <c r="F13" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="G13" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="H13" t="s">
         <v>19</v>
@@ -3307,7 +3286,7 @@
         <v>161</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -3327,10 +3306,10 @@
         <v>78</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="G14" s="12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H14" t="s">
         <v>19</v>
@@ -3342,7 +3321,7 @@
         <v>161</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -3360,10 +3339,10 @@
       </c>
       <c r="E15"/>
       <c r="F15" s="12" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="G15" s="12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H15" t="s">
         <v>19</v>
@@ -3375,7 +3354,7 @@
         <v>161</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -3393,10 +3372,10 @@
       </c>
       <c r="E16"/>
       <c r="F16" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="G16" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="H16" t="s">
         <v>19</v>
@@ -3408,7 +3387,7 @@
         <v>161</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -3445,10 +3424,10 @@
         <v>78</v>
       </c>
       <c r="F19" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="G19" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="H19" t="s">
         <v>19</v>
@@ -3460,7 +3439,7 @@
         <v>161</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -3480,10 +3459,10 @@
         <v>92</v>
       </c>
       <c r="F20" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="G20" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="H20" t="s">
         <v>19</v>
@@ -3495,7 +3474,7 @@
         <v>161</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -3515,10 +3494,10 @@
         <v>92</v>
       </c>
       <c r="F21" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="G21" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="H21" t="s">
         <v>19</v>
@@ -3530,7 +3509,7 @@
         <v>161</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -3550,10 +3529,10 @@
         <v>78</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="G22" s="12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H22" t="s">
         <v>19</v>
@@ -3565,7 +3544,7 @@
         <v>161</v>
       </c>
       <c r="K22" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -3583,10 +3562,10 @@
       </c>
       <c r="E23"/>
       <c r="F23" s="12" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="G23" s="12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H23" t="s">
         <v>19</v>
@@ -3598,7 +3577,7 @@
         <v>161</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -3616,10 +3595,10 @@
       </c>
       <c r="E24"/>
       <c r="F24" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="G24" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="H24" t="s">
         <v>19</v>
@@ -3631,7 +3610,7 @@
         <v>161</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -3681,10 +3660,10 @@
         <v>78</v>
       </c>
       <c r="F27" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="G27" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="H27" t="s">
         <v>19</v>
@@ -3696,7 +3675,7 @@
         <v>161</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -3716,10 +3695,10 @@
         <v>92</v>
       </c>
       <c r="F28" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="G28" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="H28" t="s">
         <v>19</v>
@@ -3731,7 +3710,7 @@
         <v>161</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -3751,10 +3730,10 @@
         <v>92</v>
       </c>
       <c r="F29" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="G29" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="H29" t="s">
         <v>19</v>
@@ -3766,7 +3745,7 @@
         <v>161</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -3784,10 +3763,10 @@
       </c>
       <c r="E30"/>
       <c r="F30" s="12" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="G30" s="12" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H30" t="s">
         <v>19</v>
@@ -3799,7 +3778,7 @@
         <v>161</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -3817,10 +3796,10 @@
       </c>
       <c r="E31"/>
       <c r="F31" s="12" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="G31" s="12" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="H31" t="s">
         <v>19</v>
@@ -3832,7 +3811,7 @@
         <v>161</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -3850,10 +3829,10 @@
       </c>
       <c r="E32"/>
       <c r="F32" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="G32" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="H32" t="s">
         <v>19</v>
@@ -3865,7 +3844,7 @@
         <v>161</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -4145,7 +4124,7 @@
         <v>119</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -4180,7 +4159,7 @@
         <v>119</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -4215,7 +4194,7 @@
         <v>119</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -4250,7 +4229,7 @@
         <v>119</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -4285,12 +4264,12 @@
         <v>119</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="B7" s="5">
         <v>50</v>
@@ -4302,13 +4281,13 @@
         <v>5</v>
       </c>
       <c r="E7" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="G7" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="H7" t="s">
         <v>19</v>
@@ -4317,15 +4296,15 @@
         <v>0.1</v>
       </c>
       <c r="J7" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B8" s="5">
         <v>150</v>
@@ -4337,13 +4316,13 @@
         <v>5</v>
       </c>
       <c r="E8" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="G8" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="H8" t="s">
         <v>19</v>
@@ -4352,15 +4331,15 @@
         <v>0.1</v>
       </c>
       <c r="J8" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B9" s="5">
         <v>300</v>
@@ -4372,13 +4351,13 @@
         <v>5</v>
       </c>
       <c r="E9" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="G9" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="H9" t="s">
         <v>19</v>
@@ -4387,15 +4366,15 @@
         <v>0.1</v>
       </c>
       <c r="J9" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="B10" s="5">
         <v>200</v>
@@ -4407,13 +4386,13 @@
         <v>5</v>
       </c>
       <c r="E10" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="G10" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="H10" t="s">
         <v>19</v>
@@ -4422,10 +4401,10 @@
         <v>0.1</v>
       </c>
       <c r="J10" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -4449,7 +4428,7 @@
         <v>139</v>
       </c>
       <c r="H11" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="I11">
         <v>0.05</v>
@@ -4458,7 +4437,7 @@
         <v>76</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -4493,7 +4472,7 @@
         <v>76</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -4528,7 +4507,7 @@
         <v>76</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -4563,7 +4542,7 @@
         <v>76</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -4598,7 +4577,7 @@
         <v>76</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -4633,7 +4612,7 @@
         <v>76</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -4668,7 +4647,7 @@
         <v>76</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -4703,7 +4682,7 @@
         <v>76</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -4758,7 +4737,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="B2">
         <v>0.13</v>
@@ -4770,13 +4749,13 @@
         <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="F2" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="G2" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="H2" t="s">
         <v>19</v>
@@ -4785,15 +4764,15 @@
         <v>0.01</v>
       </c>
       <c r="J2" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K2" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="B3">
         <v>0.9</v>
@@ -4805,13 +4784,13 @@
         <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="F3" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="G3" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="H3" t="s">
         <v>14</v>
@@ -4820,15 +4799,15 @@
         <v>0.05</v>
       </c>
       <c r="J3" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K3" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="B4">
         <v>0.9</v>
@@ -4840,30 +4819,30 @@
         <v>4</v>
       </c>
       <c r="E4" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="F4" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="G4" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="H4" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="I4">
         <v>0.05</v>
       </c>
       <c r="J4" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K4" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="B5">
         <v>0.5</v>
@@ -4875,13 +4854,13 @@
         <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="F5" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="G5" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="H5" t="s">
         <v>19</v>
@@ -4890,15 +4869,15 @@
         <v>0.05</v>
       </c>
       <c r="J5" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K5" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="B6">
         <v>25</v>
@@ -4910,13 +4889,13 @@
         <v>5</v>
       </c>
       <c r="E6" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="F6" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="G6" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="H6" t="s">
         <v>19</v>
@@ -4925,15 +4904,15 @@
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K6" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="B7">
         <v>15</v>
@@ -4945,13 +4924,13 @@
         <v>5</v>
       </c>
       <c r="E7" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="F7" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="G7" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="H7" t="s">
         <v>19</v>
@@ -4960,15 +4939,15 @@
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K7" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="B8">
         <v>30</v>
@@ -4980,13 +4959,13 @@
         <v>5</v>
       </c>
       <c r="E8" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="F8" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="G8" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="H8" t="s">
         <v>19</v>
@@ -4995,15 +4974,15 @@
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K8" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="B9">
         <v>40</v>
@@ -5015,13 +4994,13 @@
         <v>5</v>
       </c>
       <c r="E9" t="s">
+        <v>281</v>
+      </c>
+      <c r="F9" t="s">
         <v>288</v>
       </c>
-      <c r="F9" t="s">
-        <v>295</v>
-      </c>
       <c r="G9" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="H9" t="s">
         <v>19</v>
@@ -5030,15 +5009,15 @@
         <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K9" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="B10">
         <v>50</v>
@@ -5050,13 +5029,13 @@
         <v>5</v>
       </c>
       <c r="E10" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="F10" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="G10" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="H10" t="s">
         <v>19</v>
@@ -5065,15 +5044,15 @@
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="K10" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="B11">
         <v>0.6</v>
@@ -5085,10 +5064,10 @@
         <v>5</v>
       </c>
       <c r="F11" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="G11" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="H11" t="s">
         <v>19</v>
@@ -5100,12 +5079,12 @@
         <v>76</v>
       </c>
       <c r="K11" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="B12">
         <v>1.3</v>
@@ -5117,10 +5096,10 @@
         <v>5</v>
       </c>
       <c r="F12" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="G12" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="H12" t="s">
         <v>19</v>
@@ -5132,12 +5111,12 @@
         <v>76</v>
       </c>
       <c r="K12" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="B13">
         <v>1.4</v>
@@ -5149,10 +5128,10 @@
         <v>5</v>
       </c>
       <c r="F13" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="G13" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="H13" t="s">
         <v>19</v>
@@ -5164,12 +5143,12 @@
         <v>76</v>
       </c>
       <c r="K13" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="B14">
         <v>0.4</v>
@@ -5181,10 +5160,10 @@
         <v>5</v>
       </c>
       <c r="F14" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="G14" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="H14" t="s">
         <v>19</v>
@@ -5196,7 +5175,7 @@
         <v>76</v>
       </c>
       <c r="K14" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -5285,82 +5264,37 @@
         <v>1000</v>
       </c>
       <c r="J2" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="K2" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="L2"/>
       <c r="M2"/>
       <c r="N2"/>
     </row>
     <row r="3" spans="1:14">
-      <c r="A3" t="s">
-        <v>183</v>
-      </c>
-      <c r="B3">
-        <v>50.866</v>
-      </c>
-      <c r="C3">
-        <v>50.866</v>
-      </c>
-      <c r="D3" t="s">
-        <v>4</v>
-      </c>
+      <c r="A3"/>
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
       <c r="E3"/>
-      <c r="F3" t="s">
-        <v>184</v>
-      </c>
-      <c r="G3" t="s">
-        <v>185</v>
-      </c>
-      <c r="H3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>191</v>
-      </c>
+      <c r="F3"/>
+      <c r="G3"/>
+      <c r="H3"/>
+      <c r="I3"/>
     </row>
     <row r="4" spans="1:14">
-      <c r="A4" t="s">
-        <v>195</v>
-      </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4">
-        <v>4</v>
-      </c>
-      <c r="D4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" t="s">
-        <v>35</v>
-      </c>
-      <c r="F4" t="s">
-        <v>196</v>
-      </c>
-      <c r="G4" t="s">
-        <v>197</v>
-      </c>
-      <c r="H4" t="s">
-        <v>19</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="J4" t="s">
-        <v>193</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>191</v>
-      </c>
+      <c r="A4"/>
+      <c r="B4"/>
+      <c r="C4"/>
+      <c r="D4"/>
+      <c r="E4"/>
+      <c r="F4"/>
+      <c r="G4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+      <c r="J4"/>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="4"/>

</xml_diff>